<commit_message>
remove many-to-many relationship, add deployment notes, working prototype
</commit_message>
<xml_diff>
--- a/doc/data/sensor_tracking_BLANK.xlsx
+++ b/doc/data/sensor_tracking_BLANK.xlsx
@@ -8,10 +8,10 @@
   </bookViews>
   <sheets>
     <sheet name="location" sheetId="1" r:id="rId1"/>
-    <sheet name="link-deployment-contact" sheetId="2" r:id="rId2"/>
-    <sheet name="hotspot" sheetId="3" r:id="rId3"/>
-    <sheet name="sensor" sheetId="4" r:id="rId4"/>
-    <sheet name="registration" sheetId="5" r:id="rId5"/>
+    <sheet name="hotspot" sheetId="2" r:id="rId2"/>
+    <sheet name="sensor" sheetId="3" r:id="rId3"/>
+    <sheet name="registration" sheetId="4" r:id="rId4"/>
+    <sheet name="deployment-note" sheetId="5" r:id="rId5"/>
     <sheet name="sensor-note" sheetId="6" r:id="rId6"/>
     <sheet name="contact" sheetId="7" r:id="rId7"/>
     <sheet name="deployment" sheetId="8" r:id="rId8"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="34">
   <si>
     <t>address</t>
   </si>
@@ -41,85 +41,85 @@
     <t>longitude</t>
   </si>
   <si>
+    <t>macaddr</t>
+  </si>
+  <si>
+    <t>serialnum</t>
+  </si>
+  <si>
+    <t>status</t>
+  </si>
+  <si>
+    <t>ssid</t>
+  </si>
+  <si>
+    <t>password</t>
+  </si>
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>type</t>
+  </si>
+  <si>
+    <t>id</t>
+  </si>
+  <si>
+    <t>reg_email</t>
+  </si>
+  <si>
+    <t>outside</t>
+  </si>
+  <si>
+    <t>sensor_name</t>
+  </si>
+  <si>
+    <t>public</t>
+  </si>
+  <si>
+    <t>owner_name</t>
+  </si>
+  <si>
+    <t>owner_email</t>
+  </si>
+  <si>
+    <t>smsalert_number</t>
+  </si>
+  <si>
     <t>deployment_name</t>
   </si>
   <si>
+    <t>date</t>
+  </si>
+  <si>
+    <t>author</t>
+  </si>
+  <si>
+    <t>note</t>
+  </si>
+  <si>
+    <t>fullname</t>
+  </si>
+  <si>
+    <t>email</t>
+  </si>
+  <si>
+    <t>phone</t>
+  </si>
+  <si>
+    <t>sensor_index</t>
+  </si>
+  <si>
+    <t>start_date</t>
+  </si>
+  <si>
+    <t>end_date</t>
+  </si>
+  <si>
+    <t>location_address</t>
+  </si>
+  <si>
     <t>contact_fullname</t>
-  </si>
-  <si>
-    <t>macaddr</t>
-  </si>
-  <si>
-    <t>serialnum</t>
-  </si>
-  <si>
-    <t>status</t>
-  </si>
-  <si>
-    <t>ssid</t>
-  </si>
-  <si>
-    <t>password</t>
-  </si>
-  <si>
-    <t>name</t>
-  </si>
-  <si>
-    <t>type</t>
-  </si>
-  <si>
-    <t>id</t>
-  </si>
-  <si>
-    <t>reg_email</t>
-  </si>
-  <si>
-    <t>outside</t>
-  </si>
-  <si>
-    <t>sensor_name</t>
-  </si>
-  <si>
-    <t>public</t>
-  </si>
-  <si>
-    <t>owner_name</t>
-  </si>
-  <si>
-    <t>owner_email</t>
-  </si>
-  <si>
-    <t>smsalert_number</t>
-  </si>
-  <si>
-    <t>date</t>
-  </si>
-  <si>
-    <t>author</t>
-  </si>
-  <si>
-    <t>note</t>
-  </si>
-  <si>
-    <t>fullname</t>
-  </si>
-  <si>
-    <t>email</t>
-  </si>
-  <si>
-    <t>phone</t>
-  </si>
-  <si>
-    <t>sensor_index</t>
-  </si>
-  <si>
-    <t>start_date</t>
-  </si>
-  <si>
-    <t>end_date</t>
-  </si>
-  <si>
-    <t>location_address</t>
   </si>
   <si>
     <t>hotspot_macaddr</t>
@@ -517,28 +517,6 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -551,19 +529,19 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>10</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -571,7 +549,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D1"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -584,16 +562,16 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>8</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -601,7 +579,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:K1"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -620,22 +598,22 @@
   <sheetData>
     <row r="1" spans="1:11">
       <c r="A1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>17</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>19</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>4</v>
@@ -644,13 +622,47 @@
         <v>5</v>
       </c>
       <c r="I1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J1" s="1" t="s">
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="2.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>22</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -672,19 +684,19 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>24</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -704,13 +716,13 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -720,7 +732,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="6" bestFit="1" customWidth="1"/>
@@ -728,29 +740,32 @@
     <col min="4" max="4" width="10" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="16" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="16.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>33</v>
       </c>
     </row>

</xml_diff>